<commit_message>
Complete schema_header_2row coverage for remaining raw_header layouts.
Add vertical-merge-repeated, bidirectional-merge-rep, and mixed-merge fixtures so the 2-row header track matches all raw_header cases.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/excel/testdata/schema_header_2row/schema_header_2row_tests.xlsx
+++ b/excel/testdata/schema_header_2row/schema_header_2row_tests.xlsx
@@ -13,13 +13,16 @@
     <sheet name="2-row-vertical-merge" sheetId="4" r:id="rId7"/>
     <sheet name="2-row-bidirectional-merge" sheetId="5" r:id="rId8"/>
     <sheet name="2-row-horizontal-merge-repeated" sheetId="6" r:id="rId9"/>
+    <sheet name="2-row-vertical-merge-repeated" sheetId="7" r:id="rId10"/>
+    <sheet name="2-row-bidirectional-merge-rep" sheetId="8" r:id="rId11"/>
+    <sheet name="2-row-mixed-merge" sheetId="9" r:id="rId12"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>group1</t>
   </si>
@@ -115,6 +118,72 @@
   </si>
   <si>
     <t>r5cG</t>
+  </si>
+  <si>
+    <t>r3cH</t>
+  </si>
+  <si>
+    <t>r4cH</t>
+  </si>
+  <si>
+    <t>r5cH</t>
+  </si>
+  <si>
+    <t>r3cI</t>
+  </si>
+  <si>
+    <t>r4cI</t>
+  </si>
+  <si>
+    <t>r5cI</t>
+  </si>
+  <si>
+    <t>groupA</t>
+  </si>
+  <si>
+    <t>groupB</t>
+  </si>
+  <si>
+    <t>groupC</t>
+  </si>
+  <si>
+    <t>headerJ</t>
+  </si>
+  <si>
+    <t>headerH</t>
+  </si>
+  <si>
+    <t>headerI</t>
+  </si>
+  <si>
+    <t>headerK</t>
+  </si>
+  <si>
+    <t>r3cJ</t>
+  </si>
+  <si>
+    <t>r4cJ</t>
+  </si>
+  <si>
+    <t>r5cJ</t>
+  </si>
+  <si>
+    <t>r3cK</t>
+  </si>
+  <si>
+    <t>r4cK</t>
+  </si>
+  <si>
+    <t>r5cK</t>
+  </si>
+  <si>
+    <t>r3cL</t>
+  </si>
+  <si>
+    <t>r4cL</t>
+  </si>
+  <si>
+    <t>r5cL</t>
   </si>
 </sst>
 </file>
@@ -836,4 +905,383 @@
     <mergeCell ref="D1:F1"/>
   </mergeCells>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="C1:D2"/>
+    <mergeCell ref="F1:H2"/>
+  </mergeCells>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I1" t="s">
+        <v>40</v>
+      </c>
+      <c r="J1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I2" t="s">
+        <v>43</v>
+      </c>
+      <c r="L2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" t="s">
+        <v>32</v>
+      </c>
+      <c r="I3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" t="s">
+        <v>45</v>
+      </c>
+      <c r="K3" t="s">
+        <v>48</v>
+      </c>
+      <c r="L3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>33</v>
+      </c>
+      <c r="I4" t="s">
+        <v>36</v>
+      </c>
+      <c r="J4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K4" t="s">
+        <v>49</v>
+      </c>
+      <c r="L4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J5" t="s">
+        <v>47</v>
+      </c>
+      <c r="K5" t="s">
+        <v>50</v>
+      </c>
+      <c r="L5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="J1:K2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="G1:H1"/>
+  </mergeCells>
+</worksheet>
 </file>
</xml_diff>